<commit_message>
web/tests: restore Workday parser, tests and reload-wipe fix reverted on main
origin/main (revert of PR #35's merge) lost work that had already been
merged from the sam branch: web/lib/workday.js and its tests, the real-export
truncated-dimension regression fixture/test, hub/workday.py's read_only=False
+ dedupe-by-code fix, Terrace's oracle e2e test for the Workday-import
reload-wipe bug, and the lib/hub.js processing-layer functions (formatDue,
mergeCourses, selectActiveItems/selectVisibleItems/selectCourseItems) that
fixed it. Restoring all of it here since sam-figma builds on top.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/workday_view_my_courses.xlsx
+++ b/fixtures/workday_view_my_courses.xlsx
@@ -413,97 +413,333 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>View My Courses</t>
+          <t>My Enrolled Courses</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Enrolled Sections</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Course Listing</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Drop</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Swap</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Withdraw</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Credits</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Grading Basis</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Registration Status</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Instructional Format</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Delivery Mode</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>Meeting Patterns</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Grading Basis</t>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>End Date</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CPSC 121 001 - Models of Computation</t>
+          <t>Student (00000000) - Faculty of Fake Studies/Undergraduate - 2026-01-01 - Active - BMEG 000 - Fake Thermodynamics</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>BMEG 000 - Fake Thermodynamics</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Graded</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>BMEG 000 - Fake Thermodynamics-101 - Fake Thermodynamics</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>Lecture</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-09-08 - 2026-12-05 | Mon Wed Fri | 10:00 A.M. - 11:00 A.M. | Lecture | Detwiler Pavilion (DMP) | Floor: 1 | Room: 110</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Graded</t>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-08 - 2026-12-05 | Mon Wed Fri | 10:00 a.m. - 11:00 a.m. | Fake Building (FAKE) | Floor: 1 | Room: 100</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>J. Instructor</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MATH 200 201 - Calculus III</t>
+          <t>Student (00000000) - Faculty of Fake Studies/Undergraduate - 2026-01-01 - Active - BMEG 000 - Fake Thermodynamics</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lecture</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-09-08 - 2026-12-05 | Tue Thu | 9:30 A.M. - 11:00 A.M. | Lecture | Mathematics Building (MATX) | Floor: 2 | Room: 1100</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+          <t>BMEG 000 - Fake Thermodynamics</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>Graded</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>BMEG 000 - Fake Thermodynamics-L1A - Fake Thermodynamics</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-08 - 2026-12-05 | Mon Wed Fri | 10:00 a.m. - 11:00 a.m. | Fake Building (FAKE) | Floor: 1 | Room: 100</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>J. Instructor</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cpsc 210 - Software Construction</t>
+          <t>Student (00000000) - Faculty of Fake Studies/Undergraduate - 2026-01-01 - Active - BMEG 001 - Fake Cell Systems</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>BMEG 001 - Fake Cell Systems</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Graded</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>BMEG 001 - Fake Cell Systems-201 - Fake Cell Systems</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>Lecture</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-08 - 2026-12-05 | Mon Wed Fri | 10:00 a.m. - 11:00 a.m. | Fake Building (FAKE) | Floor: 1 | Room: 100</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>A. Professor</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Student (00000000) - Faculty of Fake Studies/Undergraduate - 2026-01-01 - Active - bmeg002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>bmeg002</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>Graded</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>bmeg002-301</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-08 - 2026-12-05 | Mon Wed Fri | 10:00 a.m. - 11:00 a.m. | Fake Building (FAKE) | Floor: 1 | Room: 100</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>A. Professor</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
         </is>
       </c>
     </row>

</xml_diff>